<commit_message>
[monitoramento 14/09] Mestra corrigida fecha a bijecao ao centavo; termos e segmentacao arquivados
A linha L61 passou a desconto 91,59 e receita 519,03, e L61/L62 ganharam STATUS
VALIDO. Soma da Mestra em 07-14/09 = R$ 1.854,36, identica ao Business Report.
Diferenca zero.

Arquivados os recorrentes de Termos e Segmentacao (janela 15/08-13/09) e a
proposta de veredito para EC-003 e EC-004.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1906" uniqueCount="562">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1951,7 +1951,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -19415,11 +19429,11 @@
         <v>203.54</v>
       </c>
       <c r="F61" s="20">
-        <v>25.95</v>
+        <v>91.59</v>
       </c>
       <c r="G61" s="13">
         <f t="shared" si="6"/>
-        <v>584.66999999999996</v>
+        <v>519.03</v>
       </c>
       <c r="H61" s="8" t="str">
         <f>IF($B61="","",INDEX(Simulador!$B$7:$B$232,MATCH($B61,Simulador!$A$7:$A$232,0)))</f>
@@ -19434,7 +19448,7 @@
       </c>
       <c r="K61" s="20">
         <f t="shared" si="11"/>
-        <v>90</v>
+        <v>81.14</v>
       </c>
       <c r="L61" s="13">
         <f>IF(OR($B61="",$C61=""),"",$C61*INDEX(Simulador!$F$7:$F$232,MATCH($B61,Simulador!$A$7:$A$232,0)))</f>
@@ -19442,22 +19456,25 @@
       </c>
       <c r="M61" s="13">
         <f t="shared" si="7"/>
-        <v>58.466999999999999</v>
+        <v>51.902999999999999</v>
       </c>
       <c r="N61" s="35">
         <f t="shared" si="8"/>
-        <v>131.88300000000004</v>
+        <v>81.667000000000058</v>
       </c>
       <c r="O61" s="12">
         <f t="shared" si="9"/>
-        <v>0.22556826928010681</v>
+        <v>0.157345432826619</v>
       </c>
       <c r="P61" s="22" t="str">
         <f t="shared" si="10"/>
-        <v>ACIMA DA META (&gt;20%)</v>
+        <v>DENTRO DA META (15-20%)</v>
       </c>
       <c r="Q61" s="19"/>
       <c r="R61" s="19"/>
+      <c r="S61" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="62" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="32">
@@ -19518,6 +19535,9 @@
       </c>
       <c r="Q62" s="19"/>
       <c r="R62" s="19"/>
+      <c r="S62" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="63" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="32"/>
@@ -21775,11 +21795,11 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>24567.500000000007</v>
+        <v>24501.860000000008</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>3736.0500000000011</v>
+        <v>3727.190000000001</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
@@ -21787,26 +21807,26 @@
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2456.7500000000005</v>
+        <v>2450.1860000000001</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6226.670000000001</v>
+        <v>6176.4540000000015</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25345151114276987</v>
+        <v>0.25208102568539692</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S60">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+  <conditionalFormatting sqref="S6:S62">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[15/09] Mestra: tres vendas novas (L1618-T 14/09, P3070 e L2025-T 15/09)
Linhas 63-65 do Registro_Vendas. Aritmetica conferida linha a linha e no
total: receita 24.501,86 -> 25.366,94 (+865,08), lucro 6.176,45 -> 6.434,96
(+258,50), margem global 25,21% -> 25,37%. As 11 validacoes de dados
seguem intactas.

Os tres SKUs sao exatamente os tres sinalizados como preocupacao no
monitoramento de 14/09 por trafego alto com zero venda: L2025-T (52
sessoes), P3070 (27) e L1618-T (26). Todos converteram em 24-48h.

Pendencia: a coluna STATUS das tres linhas esta vazia — marcar VALIDO.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1906" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1912" uniqueCount="562">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1951,21 +1951,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -19540,151 +19526,181 @@
       </c>
     </row>
     <row r="63" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="32"/>
-      <c r="B63" s="19"/>
-      <c r="C63" s="19"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="20" t="str">
+      <c r="A63" s="32">
+        <v>46279</v>
+      </c>
+      <c r="B63" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C63" s="19">
+        <v>1</v>
+      </c>
+      <c r="D63" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E63" s="20">
         <f>IF($B63="","",INDEX(Simulador!$D$7:$D$232,MATCH($B63,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="F63" s="20"/>
-      <c r="G63" s="13" t="str">
+      <c r="G63" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>116</v>
       </c>
       <c r="H63" s="8" t="str">
         <f>IF($B63="","",INDEX(Simulador!$B$7:$B$232,MATCH($B63,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I63" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I63" s="13">
         <f>IF(OR(H63="",$D63=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D63,Ref_Frete!$A$2:$A$54,0),IF(H63="Pequenos",2,IF(H63="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J63" s="20"/>
-      <c r="K63" s="20" t="str">
+        <v>12.9</v>
+      </c>
+      <c r="J63" s="20">
+        <v>10.39</v>
+      </c>
+      <c r="K63" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L63" s="13" t="str">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="L63" s="13">
         <f>IF(OR($B63="",$C63=""),"",$C63*INDEX(Simulador!$F$7:$F$232,MATCH($B63,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M63" s="13" t="str">
+        <v>54.47</v>
+      </c>
+      <c r="M63" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N63" s="35" t="str">
+        <v>11.600000000000001</v>
+      </c>
+      <c r="N63" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O63" s="12" t="str">
+        <v>35.040000000000013</v>
+      </c>
+      <c r="O63" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.30206896551724149</v>
       </c>
       <c r="P63" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q63" s="19"/>
       <c r="R63" s="19"/>
     </row>
     <row r="64" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="32"/>
-      <c r="B64" s="19"/>
-      <c r="C64" s="19"/>
-      <c r="D64" s="19"/>
-      <c r="E64" s="20" t="str">
+      <c r="A64" s="32">
+        <v>46280</v>
+      </c>
+      <c r="B64" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C64" s="19">
+        <v>1</v>
+      </c>
+      <c r="D64" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E64" s="20">
         <f>IF($B64="","",INDEX(Simulador!$D$7:$D$232,MATCH($B64,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="F64" s="20"/>
-      <c r="G64" s="13" t="str">
+      <c r="G64" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="H64" s="8" t="str">
         <f>IF($B64="","",INDEX(Simulador!$B$7:$B$232,MATCH($B64,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I64" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I64" s="13">
         <f>IF(OR(H64="",$D64=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D64,Ref_Frete!$A$2:$A$54,0),IF(H64="Pequenos",2,IF(H64="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J64" s="20"/>
-      <c r="K64" s="20" t="str">
+        <v>34.9</v>
+      </c>
+      <c r="J64" s="20">
+        <v>35.119999999999997</v>
+      </c>
+      <c r="K64" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L64" s="13" t="str">
+        <v>87.9</v>
+      </c>
+      <c r="L64" s="13">
         <f>IF(OR($B64="",$C64=""),"",$C64*INDEX(Simulador!$F$7:$F$232,MATCH($B64,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M64" s="13" t="str">
+        <v>307.26</v>
+      </c>
+      <c r="M64" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N64" s="35" t="str">
+        <v>61.617999999999995</v>
+      </c>
+      <c r="N64" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O64" s="12" t="str">
+        <v>159.18199999999996</v>
+      </c>
+      <c r="O64" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.25833684962186371</v>
       </c>
       <c r="P64" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q64" s="19"/>
       <c r="R64" s="19"/>
     </row>
     <row r="65" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="32"/>
-      <c r="B65" s="19"/>
-      <c r="C65" s="19"/>
-      <c r="D65" s="19"/>
-      <c r="E65" s="20" t="str">
+      <c r="A65" s="32">
+        <v>46280</v>
+      </c>
+      <c r="B65" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="C65" s="19">
+        <v>1</v>
+      </c>
+      <c r="D65" s="19" t="s">
+        <v>377</v>
+      </c>
+      <c r="E65" s="20">
         <f>IF($B65="","",INDEX(Simulador!$D$7:$D$232,MATCH($B65,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="F65" s="20"/>
-      <c r="G65" s="13" t="str">
+      <c r="G65" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>132.9</v>
       </c>
       <c r="H65" s="8" t="str">
         <f>IF($B65="","",INDEX(Simulador!$B$7:$B$232,MATCH($B65,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I65" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I65" s="13">
         <f>IF(OR(H65="",$D65=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D65,Ref_Frete!$A$2:$A$54,0),IF(H65="Pequenos",2,IF(H65="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J65" s="20"/>
-      <c r="K65" s="20" t="str">
+        <v>52</v>
+      </c>
+      <c r="J65" s="20">
+        <v>19.260000000000002</v>
+      </c>
+      <c r="K65" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L65" s="13" t="str">
+        <v>24.96</v>
+      </c>
+      <c r="L65" s="13">
         <f>IF(OR($B65="",$C65=""),"",$C65*INDEX(Simulador!$F$7:$F$232,MATCH($B65,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M65" s="13" t="str">
+        <v>63.11</v>
+      </c>
+      <c r="M65" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N65" s="35" t="str">
+        <v>13.290000000000001</v>
+      </c>
+      <c r="N65" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O65" s="12" t="str">
+        <v>64.28</v>
+      </c>
+      <c r="O65" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.48367193378480061</v>
       </c>
       <c r="P65" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q65" s="19"/>
       <c r="R65" s="19"/>
@@ -21795,27 +21811,27 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>24501.860000000008</v>
+        <v>25366.94000000001</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>3727.190000000001</v>
+        <v>3857.4500000000012</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>12897.240000000002</v>
+        <v>13322.080000000002</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2450.1860000000001</v>
+        <v>2536.694</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6176.4540000000015</v>
+        <v>6434.956000000001</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25208102568539692</v>
+        <v>0.25367490126913211</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -21823,10 +21839,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="S6:S62">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[15/09] Mestra: STATUS VALIDO nas linhas 63-65
Diff conferido: exatamente 3 celulas alteradas, nenhuma colateral. Nenhuma
linha com SKU ficou sem STATUS no Registro_Vendas. As 11 validacoes de
dados seguem intactas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1912" uniqueCount="562">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1915" uniqueCount="562">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1951,7 +1951,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -19584,6 +19598,9 @@
       </c>
       <c r="Q63" s="19"/>
       <c r="R63" s="19"/>
+      <c r="S63" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="64" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="32">
@@ -19644,8 +19661,11 @@
       </c>
       <c r="Q64" s="19"/>
       <c r="R64" s="19"/>
-    </row>
-    <row r="65" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S64" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="32">
         <v>46280</v>
       </c>
@@ -19704,8 +19724,11 @@
       </c>
       <c r="Q65" s="19"/>
       <c r="R65" s="19"/>
-    </row>
-    <row r="66" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="S65" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="32"/>
       <c r="B66" s="19"/>
       <c r="C66" s="19"/>
@@ -19755,7 +19778,7 @@
       <c r="Q66" s="19"/>
       <c r="R66" s="19"/>
     </row>
-    <row r="67" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="32"/>
       <c r="B67" s="19"/>
       <c r="C67" s="19"/>
@@ -19805,7 +19828,7 @@
       <c r="Q67" s="19"/>
       <c r="R67" s="19"/>
     </row>
-    <row r="68" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="32"/>
       <c r="B68" s="19"/>
       <c r="C68" s="19"/>
@@ -19855,7 +19878,7 @@
       <c r="Q68" s="19"/>
       <c r="R68" s="19"/>
     </row>
-    <row r="69" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="32"/>
       <c r="B69" s="19"/>
       <c r="C69" s="19"/>
@@ -19905,7 +19928,7 @@
       <c r="Q69" s="19"/>
       <c r="R69" s="19"/>
     </row>
-    <row r="70" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="32"/>
       <c r="B70" s="19"/>
       <c r="C70" s="19"/>
@@ -19955,7 +19978,7 @@
       <c r="Q70" s="19"/>
       <c r="R70" s="19"/>
     </row>
-    <row r="71" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="32"/>
       <c r="B71" s="19"/>
       <c r="C71" s="19"/>
@@ -20005,7 +20028,7 @@
       <c r="Q71" s="19"/>
       <c r="R71" s="19"/>
     </row>
-    <row r="72" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="32"/>
       <c r="B72" s="19"/>
       <c r="C72" s="19"/>
@@ -20055,7 +20078,7 @@
       <c r="Q72" s="19"/>
       <c r="R72" s="19"/>
     </row>
-    <row r="73" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="32"/>
       <c r="B73" s="19"/>
       <c r="C73" s="19"/>
@@ -20105,7 +20128,7 @@
       <c r="Q73" s="19"/>
       <c r="R73" s="19"/>
     </row>
-    <row r="74" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="32"/>
       <c r="B74" s="19"/>
       <c r="C74" s="19"/>
@@ -20155,7 +20178,7 @@
       <c r="Q74" s="19"/>
       <c r="R74" s="19"/>
     </row>
-    <row r="75" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="32"/>
       <c r="B75" s="19"/>
       <c r="C75" s="19"/>
@@ -20205,7 +20228,7 @@
       <c r="Q75" s="19"/>
       <c r="R75" s="19"/>
     </row>
-    <row r="76" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="32"/>
       <c r="B76" s="19"/>
       <c r="C76" s="19"/>
@@ -20255,7 +20278,7 @@
       <c r="Q76" s="19"/>
       <c r="R76" s="19"/>
     </row>
-    <row r="77" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="32"/>
       <c r="B77" s="19"/>
       <c r="C77" s="19"/>
@@ -20305,7 +20328,7 @@
       <c r="Q77" s="19"/>
       <c r="R77" s="19"/>
     </row>
-    <row r="78" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="32"/>
       <c r="B78" s="19"/>
       <c r="C78" s="19"/>
@@ -20355,7 +20378,7 @@
       <c r="Q78" s="19"/>
       <c r="R78" s="19"/>
     </row>
-    <row r="79" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="32"/>
       <c r="B79" s="19"/>
       <c r="C79" s="19"/>
@@ -20405,7 +20428,7 @@
       <c r="Q79" s="19"/>
       <c r="R79" s="19"/>
     </row>
-    <row r="80" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="32"/>
       <c r="B80" s="19"/>
       <c r="C80" s="19"/>
@@ -21838,11 +21861,11 @@
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S62">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+  <conditionalFormatting sqref="S6:S65">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[21/09] Mestra: frete real e STATUS nas linhas 66-67; suporte da GS1 acionado
Diff de exatamente 12 celulas: frete real, lucro, margem, veredito e STATUS
das duas vendas de L2025-T (19 e 20/09) mais a linha de totais. Aritmetica
conferida nas duas linhas. Validacoes intactas (11). Lucro global vai a
R$ 6.564,14, margem 25,37%.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1920" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="563">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -19749,7 +19749,9 @@
         <f>IF(OR(H66="",$D66=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D66,Ref_Frete!$A$2:$A$54,0),IF(H66="Pequenos",2,IF(H66="Medios",4,6))))</f>
         <v>24.9</v>
       </c>
-      <c r="J66" s="20"/>
+      <c r="J66" s="20">
+        <v>20.49</v>
+      </c>
       <c r="K66" s="20">
         <f t="shared" si="11"/>
         <v>21.3</v>
@@ -19762,20 +19764,23 @@
         <f t="shared" si="7"/>
         <v>13.290000000000001</v>
       </c>
-      <c r="N66" s="35" t="str">
+      <c r="N66" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O66" s="12" t="str">
+        <v>39.610000000000007</v>
+      </c>
+      <c r="O66" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.29804364183596693</v>
       </c>
       <c r="P66" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q66" s="19"/>
       <c r="R66" s="19"/>
+      <c r="S66" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="67" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="32">
@@ -19809,7 +19814,9 @@
         <f>IF(OR(H67="",$D67=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D67,Ref_Frete!$A$2:$A$54,0),IF(H67="Pequenos",2,IF(H67="Medios",4,6))))</f>
         <v>12.9</v>
       </c>
-      <c r="J67" s="20"/>
+      <c r="J67" s="20">
+        <v>22.01</v>
+      </c>
       <c r="K67" s="20">
         <f t="shared" si="11"/>
         <v>52.87</v>
@@ -19822,20 +19829,23 @@
         <f t="shared" si="7"/>
         <v>37.876000000000005</v>
       </c>
-      <c r="N67" s="35" t="str">
+      <c r="N67" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O67" s="12" t="str">
+        <v>89.574000000000041</v>
+      </c>
+      <c r="O67" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.23649276586756793</v>
       </c>
       <c r="P67" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q67" s="19"/>
       <c r="R67" s="19"/>
+      <c r="S67" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="68" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="32"/>
@@ -21859,18 +21869,18 @@
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6434.956000000001</v>
+        <v>6564.14</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.24865935560656291</v>
+        <v>0.25365127943551807</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S65">
+  <conditionalFormatting sqref="S6:S67">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>

<commit_message>
[24/09] Mestra: tres vendas novas (PXM 22/09, EGC 23/09, L1618-T 24/09) e devolucao na L62
Diff de exatamente 16 celulas de entrada no Registro_Vendas, nenhuma
colateral nas outras 8 abas:
- L68 PXM 2 un, Ceara Capital, R$ 407,08, lucro R$ 107,73 (26,5%)
- L69 EGC 1 un, SC Interior, R$ 674,62, lucro R$ 176,71 (26,2%)
- L70 L1618-T 1 un, ES Interior, R$ 116,00, lucro R$ 38,35 (33,1%)
- L62 (L1618-B 13/09, 2 un) STATUS VALIDO -> DEVOLUCAO; valores da linha
  preservados, conforme a convencao de status
Aritmetica conferida ao centavo nas tres linhas. Cache recalculado pelo
Excel. Validacoes intactas (3 + 4 x14). Lucro global R$ 6.886,93 sobre
R$ 27.076,30, margem 25,44%.

Pendencias: STATUS vazio em L68-L70; L62 sem numero do pedido na Obs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N9koFMNsQhQyNq9bqBjnBN
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1928" uniqueCount="563">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -19527,7 +19527,7 @@
       <c r="Q62" s="19"/>
       <c r="R62" s="19"/>
       <c r="S62" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="63" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -19848,151 +19848,181 @@
       </c>
     </row>
     <row r="68" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="32"/>
-      <c r="B68" s="19"/>
-      <c r="C68" s="19"/>
-      <c r="D68" s="19"/>
-      <c r="E68" s="20" t="str">
+      <c r="A68" s="32">
+        <v>46287</v>
+      </c>
+      <c r="B68" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C68" s="19">
+        <v>2</v>
+      </c>
+      <c r="D68" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="E68" s="20">
         <f>IF($B68="","",INDEX(Simulador!$D$7:$D$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>203.54</v>
       </c>
       <c r="F68" s="20"/>
-      <c r="G68" s="13" t="str">
+      <c r="G68" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>407.08</v>
       </c>
       <c r="H68" s="8" t="str">
         <f>IF($B68="","",INDEX(Simulador!$B$7:$B$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I68" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I68" s="13">
         <f>IF(OR(H68="",$D68=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D68,Ref_Frete!$A$2:$A$54,0),IF(H68="Pequenos",2,IF(H68="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J68" s="20"/>
-      <c r="K68" s="20" t="str">
+        <v>70</v>
+      </c>
+      <c r="J68" s="20">
+        <v>58.63</v>
+      </c>
+      <c r="K68" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L68" s="13" t="str">
+        <v>64.41</v>
+      </c>
+      <c r="L68" s="13">
         <f>IF(OR($B68="",$C68=""),"",$C68*INDEX(Simulador!$F$7:$F$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M68" s="13" t="str">
+        <v>205.6</v>
+      </c>
+      <c r="M68" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N68" s="35" t="str">
+        <v>40.707999999999998</v>
+      </c>
+      <c r="N68" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O68" s="12" t="str">
+        <v>107.73199999999997</v>
+      </c>
+      <c r="O68" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.26464576987324351</v>
       </c>
       <c r="P68" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q68" s="19"/>
       <c r="R68" s="19"/>
     </row>
     <row r="69" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="32"/>
-      <c r="B69" s="19"/>
-      <c r="C69" s="19"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="20" t="str">
+      <c r="A69" s="32">
+        <v>46288</v>
+      </c>
+      <c r="B69" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="C69" s="19">
+        <v>1</v>
+      </c>
+      <c r="D69" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E69" s="20">
         <f>IF($B69="","",INDEX(Simulador!$D$7:$D$232,MATCH($B69,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>674.62</v>
       </c>
       <c r="F69" s="20"/>
-      <c r="G69" s="13" t="str">
+      <c r="G69" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>674.62</v>
       </c>
       <c r="H69" s="8" t="str">
         <f>IF($B69="","",INDEX(Simulador!$B$7:$B$232,MATCH($B69,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I69" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I69" s="13">
         <f>IF(OR(H69="",$D69=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D69,Ref_Frete!$A$2:$A$54,0),IF(H69="Pequenos",2,IF(H69="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J69" s="20"/>
-      <c r="K69" s="20" t="str">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="J69" s="20">
+        <v>34.14</v>
+      </c>
+      <c r="K69" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L69" s="13" t="str">
+        <v>100.51</v>
+      </c>
+      <c r="L69" s="13">
         <f>IF(OR($B69="",$C69=""),"",$C69*INDEX(Simulador!$F$7:$F$232,MATCH($B69,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M69" s="13" t="str">
+        <v>365.7</v>
+      </c>
+      <c r="M69" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N69" s="35" t="str">
+        <v>67.462000000000003</v>
+      </c>
+      <c r="N69" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O69" s="12" t="str">
+        <v>176.70800000000003</v>
+      </c>
+      <c r="O69" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.26193709051021319</v>
       </c>
       <c r="P69" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q69" s="19"/>
       <c r="R69" s="19"/>
     </row>
     <row r="70" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="32"/>
-      <c r="B70" s="19"/>
-      <c r="C70" s="19"/>
-      <c r="D70" s="19"/>
-      <c r="E70" s="20" t="str">
+      <c r="A70" s="32">
+        <v>46289</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C70" s="19">
+        <v>1</v>
+      </c>
+      <c r="D70" s="19" t="s">
+        <v>412</v>
+      </c>
+      <c r="E70" s="20">
         <f>IF($B70="","",INDEX(Simulador!$D$7:$D$232,MATCH($B70,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="F70" s="20"/>
-      <c r="G70" s="13" t="str">
+      <c r="G70" s="13">
         <f t="shared" ref="G70:G101" si="12">IF(OR($B70="",$C70=""),"",$C70*E70-IF(F70="",0,F70))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="H70" s="8" t="str">
         <f>IF($B70="","",INDEX(Simulador!$B$7:$B$232,MATCH($B70,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I70" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I70" s="13">
         <f>IF(OR(H70="",$D70=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D70,Ref_Frete!$A$2:$A$54,0),IF(H70="Pequenos",2,IF(H70="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J70" s="20"/>
-      <c r="K70" s="20" t="str">
+        <v>29.9</v>
+      </c>
+      <c r="J70" s="20">
+        <v>21.78</v>
+      </c>
+      <c r="K70" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L70" s="13" t="str">
+        <v>19.7</v>
+      </c>
+      <c r="L70" s="13">
         <f>IF(OR($B70="",$C70=""),"",$C70*INDEX(Simulador!$F$7:$F$232,MATCH($B70,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M70" s="13" t="str">
+        <v>54.47</v>
+      </c>
+      <c r="M70" s="13">
         <f t="shared" ref="M70:M101" si="13">IF(G70="","",G70*$B$3)</f>
-        <v/>
-      </c>
-      <c r="N70" s="35" t="str">
+        <v>11.600000000000001</v>
+      </c>
+      <c r="N70" s="35">
         <f t="shared" ref="N70:N101" si="14">IF(OR(G70="",J70=""),"",G70+IF(I70="",0,I70)-J70-K70-L70-M70)</f>
-        <v/>
-      </c>
-      <c r="O70" s="12" t="str">
+        <v>38.35</v>
+      </c>
+      <c r="O70" s="12">
         <f t="shared" ref="O70:O101" si="15">IF(OR(N70="",G70=0,G70=""),"",N70/G70)</f>
-        <v/>
+        <v>0.33060344827586208</v>
       </c>
       <c r="P70" s="22" t="str">
         <f t="shared" ref="P70:P101" si="16">IF(O70="","",IF(O70&lt;0,"PREJUÍZO",IF(O70&lt;0.1,"CRÍTICO (&lt;10%)",IF(O70&lt;0.15,"ABAIXO DA META (10-15%)",IF(O70&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q70" s="19"/>
       <c r="R70" s="19"/>
@@ -21853,27 +21883,27 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>25878.600000000009</v>
+        <v>27076.30000000001</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>3931.6200000000013</v>
+        <v>4116.2400000000007</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>13574.520000000002</v>
+        <v>14200.290000000003</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2587.86</v>
+        <v>2707.63</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6564.14</v>
+        <v>6886.93</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25365127943551807</v>
+        <v>0.25435269959337126</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[24/09] Mestra: STATUS VALIDO em L68-L70 e pedido da devolucao na L62
Diff de exatamente 4 celulas no Registro_Vendas, nenhuma colateral:
- S68, S69, S70: VALIDO
- Q62: numero do pedido 702-4604095-6119462 (devolucao de L1618-B 13/09)
Nenhuma linha com SKU fica sem STATUS. Validacoes intactas (3 + 4 x14).
Totais inalterados: R$ 27.076,30 de receita, R$ 6.886,93 de lucro, 25,44%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N9koFMNsQhQyNq9bqBjnBN
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1928" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="564">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1724,6 +1724,9 @@
   </si>
   <si>
     <t>701-5825355-7110610 - devolução aprovada 17/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">702-4604095-6119462 </t>
   </si>
 </sst>
 </file>
@@ -1954,7 +1957,35 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -19075,7 +19106,6 @@
         <f t="shared" si="10"/>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
-      <c r="Q55" s="19"/>
       <c r="R55" s="19"/>
       <c r="S55" t="s">
         <v>560</v>
@@ -19524,7 +19554,9 @@
         <f t="shared" si="10"/>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
-      <c r="Q62" s="19"/>
+      <c r="Q62" s="19" t="s">
+        <v>563</v>
+      </c>
       <c r="R62" s="19"/>
       <c r="S62" t="s">
         <v>558</v>
@@ -19906,6 +19938,9 @@
       </c>
       <c r="Q68" s="19"/>
       <c r="R68" s="19"/>
+      <c r="S68" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="69" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="32">
@@ -19966,6 +20001,9 @@
       </c>
       <c r="Q69" s="19"/>
       <c r="R69" s="19"/>
+      <c r="S69" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="70" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="32">
@@ -20026,6 +20064,9 @@
       </c>
       <c r="Q70" s="19"/>
       <c r="R70" s="19"/>
+      <c r="S70" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="71" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="32"/>
@@ -21910,7 +21951,7 @@
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S67">
+  <conditionalFormatting sqref="S6:S70">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>

<commit_message>
[24/09] Mestra: desconto no preco (5%, EC) na venda de 2 PXM de 22/09
Diff de exatamente 1 celula de entrada: F68 = 20,36 (5% sobre 203,54,
arredondado por unidade: 10,18 x 2). Recalculo pelas formulas: receita
407,08 -> 386,72, tarifa 64,41 -> 61,66, lucro 107,73 -> 92,16, margem
26,5% -> 23,8%. Primeira venda com desconto no preco em SKU anunciado:
atribuicao Ads a conferir pedido a pedido na leitura de 28/09.
Totais: R$ 27.055,94 de receita, R$ 6.871,36 de lucro, 25,40%.
Validacoes intactas (3 + 4 x14).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N9koFMNsQhQyNq9bqBjnBN
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -1957,35 +1957,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -19896,10 +19868,12 @@
         <f>IF($B68="","",INDEX(Simulador!$D$7:$D$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
         <v>203.54</v>
       </c>
-      <c r="F68" s="20"/>
+      <c r="F68" s="20">
+        <v>20.36</v>
+      </c>
       <c r="G68" s="13">
         <f t="shared" si="6"/>
-        <v>407.08</v>
+        <v>386.71999999999997</v>
       </c>
       <c r="H68" s="8" t="str">
         <f>IF($B68="","",INDEX(Simulador!$B$7:$B$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
@@ -19914,7 +19888,7 @@
       </c>
       <c r="K68" s="20">
         <f t="shared" si="11"/>
-        <v>64.41</v>
+        <v>61.66</v>
       </c>
       <c r="L68" s="13">
         <f>IF(OR($B68="",$C68=""),"",$C68*INDEX(Simulador!$F$7:$F$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
@@ -19922,15 +19896,15 @@
       </c>
       <c r="M68" s="13">
         <f t="shared" si="7"/>
-        <v>40.707999999999998</v>
+        <v>38.671999999999997</v>
       </c>
       <c r="N68" s="35">
         <f t="shared" si="8"/>
-        <v>107.73199999999997</v>
+        <v>92.157999999999959</v>
       </c>
       <c r="O68" s="12">
         <f t="shared" si="9"/>
-        <v>0.26464576987324351</v>
+        <v>0.23830678527099702</v>
       </c>
       <c r="P68" s="22" t="str">
         <f t="shared" si="10"/>
@@ -21924,11 +21898,11 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>27076.30000000001</v>
+        <v>27055.94000000001</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4116.2400000000007</v>
+        <v>4113.4900000000016</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
@@ -21936,15 +21910,15 @@
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2707.63</v>
+        <v>2705.5940000000001</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6886.93</v>
+        <v>6871.3560000000007</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25435269959337126</v>
+        <v>0.25396848159775631</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[Monitoramento 28/09] regra de atribuicao do desconto no preco confirmada (preco com desconto; promo de quantidade empilha e nao aparece); Mestra recebida com 3 linhas a corrigir; linha 14 do Controle proposta
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1938" uniqueCount="564">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1724,6 +1724,9 @@
   </si>
   <si>
     <t>701-5825355-7110610 - devolução aprovada 17/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">702-4604095-6119462 </t>
   </si>
 </sst>
 </file>
@@ -1954,7 +1957,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -19075,7 +19092,6 @@
         <f t="shared" si="10"/>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
-      <c r="Q55" s="19"/>
       <c r="R55" s="19"/>
       <c r="S55" t="s">
         <v>560</v>
@@ -19524,10 +19540,12 @@
         <f t="shared" si="10"/>
         <v>ACIMA DA META (&gt;20%)</v>
       </c>
-      <c r="Q62" s="19"/>
+      <c r="Q62" s="19" t="s">
+        <v>563</v>
+      </c>
       <c r="R62" s="19"/>
       <c r="S62" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
     </row>
     <row r="63" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -19848,239 +19866,305 @@
       </c>
     </row>
     <row r="68" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="32"/>
-      <c r="B68" s="19"/>
-      <c r="C68" s="19"/>
-      <c r="D68" s="19"/>
-      <c r="E68" s="20" t="str">
+      <c r="A68" s="32">
+        <v>46287</v>
+      </c>
+      <c r="B68" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C68" s="19">
+        <v>2</v>
+      </c>
+      <c r="D68" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="E68" s="20">
         <f>IF($B68="","",INDEX(Simulador!$D$7:$D$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F68" s="20"/>
-      <c r="G68" s="13" t="str">
+        <v>203.54</v>
+      </c>
+      <c r="F68" s="20">
+        <v>20.36</v>
+      </c>
+      <c r="G68" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>386.71999999999997</v>
       </c>
       <c r="H68" s="8" t="str">
         <f>IF($B68="","",INDEX(Simulador!$B$7:$B$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I68" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I68" s="13">
         <f>IF(OR(H68="",$D68=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D68,Ref_Frete!$A$2:$A$54,0),IF(H68="Pequenos",2,IF(H68="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J68" s="20"/>
-      <c r="K68" s="20" t="str">
+        <v>70</v>
+      </c>
+      <c r="J68" s="20">
+        <v>58.63</v>
+      </c>
+      <c r="K68" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L68" s="13" t="str">
+        <v>61.66</v>
+      </c>
+      <c r="L68" s="13">
         <f>IF(OR($B68="",$C68=""),"",$C68*INDEX(Simulador!$F$7:$F$232,MATCH($B68,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M68" s="13" t="str">
+        <v>205.6</v>
+      </c>
+      <c r="M68" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N68" s="35" t="str">
+        <v>38.671999999999997</v>
+      </c>
+      <c r="N68" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O68" s="12" t="str">
+        <v>92.157999999999959</v>
+      </c>
+      <c r="O68" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.23830678527099702</v>
       </c>
       <c r="P68" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q68" s="19"/>
       <c r="R68" s="19"/>
+      <c r="S68" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="69" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="32"/>
-      <c r="B69" s="19"/>
-      <c r="C69" s="19"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="20" t="str">
+      <c r="A69" s="32">
+        <v>46288</v>
+      </c>
+      <c r="B69" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="C69" s="19">
+        <v>1</v>
+      </c>
+      <c r="D69" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E69" s="20">
         <f>IF($B69="","",INDEX(Simulador!$D$7:$D$232,MATCH($B69,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>674.62</v>
       </c>
       <c r="F69" s="20"/>
-      <c r="G69" s="13" t="str">
+      <c r="G69" s="13">
         <f t="shared" si="6"/>
-        <v/>
+        <v>674.62</v>
       </c>
       <c r="H69" s="8" t="str">
         <f>IF($B69="","",INDEX(Simulador!$B$7:$B$232,MATCH($B69,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I69" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I69" s="13">
         <f>IF(OR(H69="",$D69=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D69,Ref_Frete!$A$2:$A$54,0),IF(H69="Pequenos",2,IF(H69="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J69" s="20"/>
-      <c r="K69" s="20" t="str">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="J69" s="20">
+        <v>34.14</v>
+      </c>
+      <c r="K69" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L69" s="13" t="str">
+        <v>100.51</v>
+      </c>
+      <c r="L69" s="13">
         <f>IF(OR($B69="",$C69=""),"",$C69*INDEX(Simulador!$F$7:$F$232,MATCH($B69,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M69" s="13" t="str">
+        <v>365.7</v>
+      </c>
+      <c r="M69" s="13">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="N69" s="35" t="str">
+        <v>67.462000000000003</v>
+      </c>
+      <c r="N69" s="35">
         <f t="shared" si="8"/>
-        <v/>
-      </c>
-      <c r="O69" s="12" t="str">
+        <v>176.70800000000003</v>
+      </c>
+      <c r="O69" s="12">
         <f t="shared" si="9"/>
-        <v/>
+        <v>0.26193709051021319</v>
       </c>
       <c r="P69" s="22" t="str">
         <f t="shared" si="10"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q69" s="19"/>
       <c r="R69" s="19"/>
+      <c r="S69" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="70" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="32"/>
-      <c r="B70" s="19"/>
-      <c r="C70" s="19"/>
-      <c r="D70" s="19"/>
-      <c r="E70" s="20" t="str">
+      <c r="A70" s="32">
+        <v>46289</v>
+      </c>
+      <c r="B70" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C70" s="19">
+        <v>1</v>
+      </c>
+      <c r="D70" s="19" t="s">
+        <v>412</v>
+      </c>
+      <c r="E70" s="20">
         <f>IF($B70="","",INDEX(Simulador!$D$7:$D$232,MATCH($B70,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="F70" s="20"/>
-      <c r="G70" s="13" t="str">
+      <c r="G70" s="13">
         <f t="shared" ref="G70:G101" si="12">IF(OR($B70="",$C70=""),"",$C70*E70-IF(F70="",0,F70))</f>
-        <v/>
+        <v>116</v>
       </c>
       <c r="H70" s="8" t="str">
         <f>IF($B70="","",INDEX(Simulador!$B$7:$B$232,MATCH($B70,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I70" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I70" s="13">
         <f>IF(OR(H70="",$D70=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D70,Ref_Frete!$A$2:$A$54,0),IF(H70="Pequenos",2,IF(H70="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J70" s="20"/>
-      <c r="K70" s="20" t="str">
+        <v>29.9</v>
+      </c>
+      <c r="J70" s="20">
+        <v>21.78</v>
+      </c>
+      <c r="K70" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L70" s="13" t="str">
+        <v>19.7</v>
+      </c>
+      <c r="L70" s="13">
         <f>IF(OR($B70="",$C70=""),"",$C70*INDEX(Simulador!$F$7:$F$232,MATCH($B70,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M70" s="13" t="str">
+        <v>54.47</v>
+      </c>
+      <c r="M70" s="13">
         <f t="shared" ref="M70:M101" si="13">IF(G70="","",G70*$B$3)</f>
-        <v/>
-      </c>
-      <c r="N70" s="35" t="str">
+        <v>11.600000000000001</v>
+      </c>
+      <c r="N70" s="35">
         <f t="shared" ref="N70:N101" si="14">IF(OR(G70="",J70=""),"",G70+IF(I70="",0,I70)-J70-K70-L70-M70)</f>
-        <v/>
-      </c>
-      <c r="O70" s="12" t="str">
+        <v>38.35</v>
+      </c>
+      <c r="O70" s="12">
         <f t="shared" ref="O70:O101" si="15">IF(OR(N70="",G70=0,G70=""),"",N70/G70)</f>
-        <v/>
+        <v>0.33060344827586208</v>
       </c>
       <c r="P70" s="22" t="str">
         <f t="shared" ref="P70:P101" si="16">IF(O70="","",IF(O70&lt;0,"PREJUÍZO",IF(O70&lt;0.1,"CRÍTICO (&lt;10%)",IF(O70&lt;0.15,"ABAIXO DA META (10-15%)",IF(O70&lt;=0.2,"DENTRO DA META (15-20%)","ACIMA DA META (&gt;20%)")))))</f>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q70" s="19"/>
       <c r="R70" s="19"/>
+      <c r="S70" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="71" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="32"/>
-      <c r="B71" s="19"/>
-      <c r="C71" s="19"/>
-      <c r="D71" s="19"/>
-      <c r="E71" s="20" t="str">
+      <c r="A71" s="32">
+        <v>46289</v>
+      </c>
+      <c r="B71" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C71" s="19">
+        <v>3</v>
+      </c>
+      <c r="D71" s="19" t="s">
+        <v>411</v>
+      </c>
+      <c r="E71" s="20">
         <f>IF($B71="","",INDEX(Simulador!$D$7:$D$232,MATCH($B71,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F71" s="20"/>
-      <c r="G71" s="13" t="str">
+        <v>203.54</v>
+      </c>
+      <c r="F71" s="20">
+        <v>29</v>
+      </c>
+      <c r="G71" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>581.62</v>
       </c>
       <c r="H71" s="8" t="str">
         <f>IF($B71="","",INDEX(Simulador!$B$7:$B$232,MATCH($B71,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I71" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I71" s="13">
         <f>IF(OR(H71="",$D71=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D71,Ref_Frete!$A$2:$A$54,0),IF(H71="Pequenos",2,IF(H71="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J71" s="20"/>
-      <c r="K71" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J71" s="20">
+        <v>48.63</v>
+      </c>
+      <c r="K71" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L71" s="13" t="str">
+        <v>81.88</v>
+      </c>
+      <c r="L71" s="13">
         <f>IF(OR($B71="",$C71=""),"",$C71*INDEX(Simulador!$F$7:$F$232,MATCH($B71,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M71" s="13" t="str">
+        <v>308.39999999999998</v>
+      </c>
+      <c r="M71" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N71" s="35" t="str">
+        <v>58.162000000000006</v>
+      </c>
+      <c r="N71" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O71" s="12" t="str">
+        <v>109.44800000000001</v>
+      </c>
+      <c r="O71" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.18817784807950208</v>
       </c>
       <c r="P71" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>DENTRO DA META (15-20%)</v>
       </c>
       <c r="Q71" s="19"/>
       <c r="R71" s="19"/>
+      <c r="S71" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="72" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="32"/>
-      <c r="B72" s="19"/>
-      <c r="C72" s="19"/>
-      <c r="D72" s="19"/>
-      <c r="E72" s="20" t="str">
+      <c r="A72" s="32">
+        <v>46291</v>
+      </c>
+      <c r="B72" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C72" s="19">
+        <v>1</v>
+      </c>
+      <c r="D72" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="E72" s="20">
         <f>IF($B72="","",INDEX(Simulador!$D$7:$D$232,MATCH($B72,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F72" s="20"/>
-      <c r="G72" s="13" t="str">
+        <v>116</v>
+      </c>
+      <c r="F72" s="20">
+        <v>6.2</v>
+      </c>
+      <c r="G72" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>109.8</v>
       </c>
       <c r="H72" s="8" t="str">
         <f>IF($B72="","",INDEX(Simulador!$B$7:$B$232,MATCH($B72,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I72" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I72" s="13">
         <f>IF(OR(H72="",$D72=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D72,Ref_Frete!$A$2:$A$54,0),IF(H72="Pequenos",2,IF(H72="Medios",4,6))))</f>
-        <v/>
+        <v>24.9</v>
       </c>
       <c r="J72" s="20"/>
-      <c r="K72" s="20" t="str">
+      <c r="K72" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L72" s="13" t="str">
+        <v>18.18</v>
+      </c>
+      <c r="L72" s="13">
         <f>IF(OR($B72="",$C72=""),"",$C72*INDEX(Simulador!$F$7:$F$232,MATCH($B72,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M72" s="13" t="str">
+        <v>54.47</v>
+      </c>
+      <c r="M72" s="13">
         <f t="shared" si="13"/>
-        <v/>
+        <v>10.98</v>
       </c>
       <c r="N72" s="35" t="str">
         <f t="shared" si="14"/>
@@ -20096,6 +20180,9 @@
       </c>
       <c r="Q72" s="19"/>
       <c r="R72" s="19"/>
+      <c r="S72" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="73" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="32"/>
@@ -21853,38 +21940,38 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>25878.600000000009</v>
+        <v>27747.360000000008</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>3931.6200000000013</v>
+        <v>4213.550000000002</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>13574.520000000002</v>
+        <v>14563.160000000002</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2587.86</v>
+        <v>2774.7359999999999</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6564.14</v>
+        <v>6980.804000000001</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25365127943551807</v>
+        <v>0.25158443902410893</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S67">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="S6:S72">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[Monitoramento 28/09] Mestra: frete real do L1618-T de 26/09 lancado (linha 72 fechada; lucro 6.987,49, margem 25,22%)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -20141,7 +20141,9 @@
         <f>IF(OR(H72="",$D72=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D72,Ref_Frete!$A$2:$A$54,0),IF(H72="Pequenos",2,IF(H72="Medios",4,6))))</f>
         <v>24.9</v>
       </c>
-      <c r="J72" s="20"/>
+      <c r="J72" s="20">
+        <v>16.89</v>
+      </c>
       <c r="K72" s="20">
         <f t="shared" si="11"/>
         <v>18.239999999999998</v>
@@ -20154,17 +20156,17 @@
         <f t="shared" si="13"/>
         <v>11.020000000000001</v>
       </c>
-      <c r="N72" s="35" t="str">
+      <c r="N72" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O72" s="12" t="str">
+        <v>34.479999999999997</v>
+      </c>
+      <c r="O72" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.31288566243194188</v>
       </c>
       <c r="P72" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q72" s="19"/>
       <c r="R72" s="19"/>
@@ -21944,11 +21946,11 @@
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6953.0080000000007</v>
+        <v>6987.4880000000003</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25090767632983074</v>
+        <v>0.25215192869943137</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
[30/09] Mestra: 3 vendas novas (L2030-B, L1623-T 1a venda, PG4080 1a venda) a preco de tabela; totais 28.628,64 / 25,46%
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1938" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="564">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -1957,7 +1957,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -20175,154 +20189,193 @@
       </c>
     </row>
     <row r="73" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="32"/>
-      <c r="B73" s="19"/>
-      <c r="C73" s="19"/>
-      <c r="D73" s="19"/>
-      <c r="E73" s="20" t="str">
+      <c r="A73" s="32">
+        <v>46293</v>
+      </c>
+      <c r="B73" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="C73" s="19">
+        <v>1</v>
+      </c>
+      <c r="D73" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="E73" s="20">
         <f>IF($B73="","",INDEX(Simulador!$D$7:$D$232,MATCH($B73,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>153.72</v>
       </c>
       <c r="F73" s="20"/>
-      <c r="G73" s="13" t="str">
+      <c r="G73" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>153.72</v>
       </c>
       <c r="H73" s="8" t="str">
         <f>IF($B73="","",INDEX(Simulador!$B$7:$B$232,MATCH($B73,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I73" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I73" s="13">
         <f>IF(OR(H73="",$D73=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D73,Ref_Frete!$A$2:$A$54,0),IF(H73="Pequenos",2,IF(H73="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J73" s="20"/>
-      <c r="K73" s="20" t="str">
+        <v>29.9</v>
+      </c>
+      <c r="J73" s="20">
+        <v>23.87</v>
+      </c>
+      <c r="K73" s="20">
         <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="L73" s="13" t="str">
+        <v>24.79</v>
+      </c>
+      <c r="L73" s="13">
         <f>IF(OR($B73="",$C73=""),"",$C73*INDEX(Simulador!$F$7:$F$232,MATCH($B73,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M73" s="13" t="str">
+        <v>75.680000000000007</v>
+      </c>
+      <c r="M73" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N73" s="35" t="str">
+        <v>15.372</v>
+      </c>
+      <c r="N73" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O73" s="12" t="str">
+        <v>43.908000000000001</v>
+      </c>
+      <c r="O73" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.28563622170179548</v>
       </c>
       <c r="P73" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q73" s="19"/>
       <c r="R73" s="19"/>
+      <c r="S73" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="74" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="32"/>
-      <c r="B74" s="19"/>
-      <c r="C74" s="19"/>
-      <c r="D74" s="19"/>
-      <c r="E74" s="20" t="str">
+      <c r="A74" s="32">
+        <v>46293</v>
+      </c>
+      <c r="B74" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C74" s="19">
+        <v>1</v>
+      </c>
+      <c r="D74" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="E74" s="20">
         <f>IF($B74="","",INDEX(Simulador!$D$7:$D$232,MATCH($B74,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>123.93</v>
       </c>
       <c r="F74" s="20"/>
-      <c r="G74" s="13" t="str">
+      <c r="G74" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>123.93</v>
       </c>
       <c r="H74" s="8" t="str">
         <f>IF($B74="","",INDEX(Simulador!$B$7:$B$232,MATCH($B74,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I74" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I74" s="13">
         <f>IF(OR(H74="",$D74=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D74,Ref_Frete!$A$2:$A$54,0),IF(H74="Pequenos",2,IF(H74="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J74" s="20"/>
-      <c r="K74" s="20" t="str">
+        <v>12.9</v>
+      </c>
+      <c r="J74" s="20">
+        <v>12.87</v>
+      </c>
+      <c r="K74" s="20">
         <f t="shared" ref="K74:K107" si="17">IF(G74="","",ROUND($D$3*(G74+IF(I74="",0,I74)),2))</f>
-        <v/>
-      </c>
-      <c r="L74" s="13" t="str">
+        <v>18.47</v>
+      </c>
+      <c r="L74" s="13">
         <f>IF(OR($B74="",$C74=""),"",$C74*INDEX(Simulador!$F$7:$F$232,MATCH($B74,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M74" s="13" t="str">
+        <v>59.8</v>
+      </c>
+      <c r="M74" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N74" s="35" t="str">
+        <v>12.393000000000001</v>
+      </c>
+      <c r="N74" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O74" s="12" t="str">
+        <v>33.297000000000011</v>
+      </c>
+      <c r="O74" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.26867586540789162</v>
       </c>
       <c r="P74" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q74" s="19"/>
       <c r="R74" s="19"/>
+      <c r="S74" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="75" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="32"/>
-      <c r="B75" s="19"/>
-      <c r="C75" s="19"/>
-      <c r="D75" s="19"/>
-      <c r="E75" s="20" t="str">
+      <c r="A75" s="32">
+        <v>46295</v>
+      </c>
+      <c r="B75" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="C75" s="19">
+        <v>1</v>
+      </c>
+      <c r="D75" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="E75" s="20">
         <f>IF($B75="","",INDEX(Simulador!$D$7:$D$232,MATCH($B75,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>639.57000000000005</v>
       </c>
       <c r="F75" s="20"/>
-      <c r="G75" s="13" t="str">
+      <c r="G75" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>639.57000000000005</v>
       </c>
       <c r="H75" s="8" t="str">
         <f>IF($B75="","",INDEX(Simulador!$B$7:$B$232,MATCH($B75,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I75" s="13" t="str">
+        <v>Grandes</v>
+      </c>
+      <c r="I75" s="13">
         <f>IF(OR(H75="",$D75=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D75,Ref_Frete!$A$2:$A$54,0),IF(H75="Pequenos",2,IF(H75="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J75" s="20"/>
-      <c r="K75" s="20" t="str">
+        <v>274</v>
+      </c>
+      <c r="J75" s="20">
+        <v>171.55</v>
+      </c>
+      <c r="K75" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L75" s="13" t="str">
+        <v>123.33</v>
+      </c>
+      <c r="L75" s="13">
         <f>IF(OR($B75="",$C75=""),"",$C75*INDEX(Simulador!$F$7:$F$232,MATCH($B75,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M75" s="13" t="str">
+        <v>329.27</v>
+      </c>
+      <c r="M75" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N75" s="35" t="str">
+        <v>63.957000000000008</v>
+      </c>
+      <c r="N75" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O75" s="12" t="str">
+        <v>225.46299999999997</v>
+      </c>
+      <c r="O75" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.35252278874869042</v>
       </c>
       <c r="P75" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q75" s="19"/>
       <c r="R75" s="19"/>
+      <c r="S75" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="76" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="32"/>
@@ -21930,38 +21983,38 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>27711.420000000013</v>
+        <v>28628.640000000014</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4208.7000000000016</v>
+        <v>4375.2900000000018</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>14563.160000000002</v>
+        <v>15027.910000000002</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2771.1420000000003</v>
+        <v>2862.864</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>6987.4880000000003</v>
+        <v>7290.1559999999999</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25215192869943137</v>
+        <v>0.25464555773519093</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S72">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+  <conditionalFormatting sqref="S6:S75">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[30/09] Mestra corrigida: venda de 30/09 e P4080 (R$ 1.070,17), nao PG4080; totais 29.059,24 / 25,45%
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -1957,21 +1957,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -20319,7 +20305,7 @@
         <v>46295</v>
       </c>
       <c r="B75" s="19" t="s">
-        <v>183</v>
+        <v>61</v>
       </c>
       <c r="C75" s="19">
         <v>1</v>
@@ -20329,12 +20315,12 @@
       </c>
       <c r="E75" s="20">
         <f>IF($B75="","",INDEX(Simulador!$D$7:$D$232,MATCH($B75,Simulador!$A$7:$A$232,0)))</f>
-        <v>639.57000000000005</v>
+        <v>1070.17</v>
       </c>
       <c r="F75" s="20"/>
       <c r="G75" s="13">
         <f t="shared" si="12"/>
-        <v>639.57000000000005</v>
+        <v>1070.17</v>
       </c>
       <c r="H75" s="8" t="str">
         <f>IF($B75="","",INDEX(Simulador!$B$7:$B$232,MATCH($B75,Simulador!$A$7:$A$232,0)))</f>
@@ -20349,23 +20335,23 @@
       </c>
       <c r="K75" s="20">
         <f t="shared" si="17"/>
-        <v>123.33</v>
+        <v>181.46</v>
       </c>
       <c r="L75" s="13">
         <f>IF(OR($B75="",$C75=""),"",$C75*INDEX(Simulador!$F$7:$F$232,MATCH($B75,Simulador!$A$7:$A$232,0)))</f>
-        <v>329.27</v>
+        <v>553.79</v>
       </c>
       <c r="M75" s="13">
         <f t="shared" si="13"/>
-        <v>63.957000000000008</v>
+        <v>107.01700000000001</v>
       </c>
       <c r="N75" s="35">
         <f t="shared" si="14"/>
-        <v>225.46299999999997</v>
+        <v>330.35300000000012</v>
       </c>
       <c r="O75" s="12">
         <f t="shared" si="15"/>
-        <v>0.35252278874869042</v>
+        <v>0.30869207695973544</v>
       </c>
       <c r="P75" s="22" t="str">
         <f t="shared" si="16"/>
@@ -21983,27 +21969,27 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>28628.640000000014</v>
+        <v>29059.240000000013</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4375.2900000000018</v>
+        <v>4433.4200000000019</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>15027.910000000002</v>
+        <v>15252.43</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2862.864</v>
+        <v>2905.924</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>7290.1559999999999</v>
+        <v>7395.0460000000003</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.25464555773519093</v>
+        <v>0.2544817414357704</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -22011,10 +21997,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="S6:S75">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"VÁLIDO"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
[01/10] Mestra: 3 vendas novas a preco cheio (P3070, P3060 x2, PXM x3) — semana de preco limpo com 9 un; diff conferido, validacoes intactas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
+++ b/dados/Planilha_Mestra_Winnet_v4_3_4.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1947" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1956" uniqueCount="564">
   <si>
     <t>PLANILHA MESTRA WINNET — precificação, margem e frete em um lugar só</t>
   </si>
@@ -20364,154 +20364,195 @@
       </c>
     </row>
     <row r="76" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="32"/>
-      <c r="B76" s="19"/>
-      <c r="C76" s="19"/>
-      <c r="D76" s="19"/>
-      <c r="E76" s="20" t="str">
+      <c r="A76" s="32">
+        <v>46295</v>
+      </c>
+      <c r="B76" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C76" s="19">
+        <v>1</v>
+      </c>
+      <c r="D76" s="19" t="s">
+        <v>409</v>
+      </c>
+      <c r="E76" s="20">
         <f>IF($B76="","",INDEX(Simulador!$D$7:$D$232,MATCH($B76,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="F76" s="20"/>
-      <c r="G76" s="13" t="str">
+      <c r="G76" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>616.17999999999995</v>
       </c>
       <c r="H76" s="8" t="str">
         <f>IF($B76="","",INDEX(Simulador!$B$7:$B$232,MATCH($B76,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I76" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I76" s="13">
         <f>IF(OR(H76="",$D76=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D76,Ref_Frete!$A$2:$A$54,0),IF(H76="Pequenos",2,IF(H76="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J76" s="20"/>
-      <c r="K76" s="20" t="str">
+        <v>59.9</v>
+      </c>
+      <c r="J76" s="20">
+        <v>55.56</v>
+      </c>
+      <c r="K76" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L76" s="13" t="str">
+        <v>91.27</v>
+      </c>
+      <c r="L76" s="13">
         <f>IF(OR($B76="",$C76=""),"",$C76*INDEX(Simulador!$F$7:$F$232,MATCH($B76,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M76" s="13" t="str">
+        <v>307.26</v>
+      </c>
+      <c r="M76" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N76" s="35" t="str">
+        <v>61.617999999999995</v>
+      </c>
+      <c r="N76" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O76" s="12" t="str">
+        <v>160.37200000000001</v>
+      </c>
+      <c r="O76" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.26026810347625701</v>
       </c>
       <c r="P76" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q76" s="19"/>
       <c r="R76" s="19"/>
+      <c r="S76" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="77" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="32"/>
-      <c r="B77" s="19"/>
-      <c r="C77" s="19"/>
-      <c r="D77" s="19"/>
-      <c r="E77" s="20" t="str">
+      <c r="A77" s="32">
+        <v>46296</v>
+      </c>
+      <c r="B77" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C77" s="19">
+        <v>2</v>
+      </c>
+      <c r="D77" s="19" t="s">
+        <v>410</v>
+      </c>
+      <c r="E77" s="20">
         <f>IF($B77="","",INDEX(Simulador!$D$7:$D$232,MATCH($B77,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
+        <v>511.42</v>
       </c>
       <c r="F77" s="20"/>
-      <c r="G77" s="13" t="str">
+      <c r="G77" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>1022.84</v>
       </c>
       <c r="H77" s="8" t="str">
         <f>IF($B77="","",INDEX(Simulador!$B$7:$B$232,MATCH($B77,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I77" s="13" t="str">
+        <v>Medios</v>
+      </c>
+      <c r="I77" s="13">
         <f>IF(OR(H77="",$D77=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D77,Ref_Frete!$A$2:$A$54,0),IF(H77="Pequenos",2,IF(H77="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J77" s="20"/>
-      <c r="K77" s="20" t="str">
+        <v>69.900000000000006</v>
+      </c>
+      <c r="J77" s="20">
+        <v>128.4</v>
+      </c>
+      <c r="K77" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L77" s="13" t="str">
+        <v>147.52000000000001</v>
+      </c>
+      <c r="L77" s="13">
         <f>IF(OR($B77="",$C77=""),"",$C77*INDEX(Simulador!$F$7:$F$232,MATCH($B77,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M77" s="13" t="str">
+        <v>484.52</v>
+      </c>
+      <c r="M77" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N77" s="35" t="str">
+        <v>102.28400000000001</v>
+      </c>
+      <c r="N77" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O77" s="12" t="str">
+        <v>230.01600000000008</v>
+      </c>
+      <c r="O77" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.22487974658793172</v>
       </c>
       <c r="P77" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>ACIMA DA META (&gt;20%)</v>
       </c>
       <c r="Q77" s="19"/>
       <c r="R77" s="19"/>
+      <c r="S77" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="78" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="32"/>
-      <c r="B78" s="19"/>
-      <c r="C78" s="19"/>
-      <c r="D78" s="19"/>
-      <c r="E78" s="20" t="str">
+      <c r="A78" s="32">
+        <v>46296</v>
+      </c>
+      <c r="B78" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C78" s="19">
+        <v>3</v>
+      </c>
+      <c r="D78" s="19" t="s">
+        <v>411</v>
+      </c>
+      <c r="E78" s="20">
         <f>IF($B78="","",INDEX(Simulador!$D$7:$D$232,MATCH($B78,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="F78" s="20"/>
-      <c r="G78" s="13" t="str">
+        <v>203.54</v>
+      </c>
+      <c r="F78" s="20">
+        <v>30.53</v>
+      </c>
+      <c r="G78" s="13">
         <f t="shared" si="12"/>
-        <v/>
+        <v>580.09</v>
       </c>
       <c r="H78" s="8" t="str">
         <f>IF($B78="","",INDEX(Simulador!$B$7:$B$232,MATCH($B78,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="I78" s="13" t="str">
+        <v>Pequenos</v>
+      </c>
+      <c r="I78" s="13">
         <f>IF(OR(H78="",$D78=""),"",INDEX(Ref_Frete!$B$2:$G$54,MATCH($D78,Ref_Frete!$A$2:$A$54,0),IF(H78="Pequenos",2,IF(H78="Medios",4,6))))</f>
-        <v/>
-      </c>
-      <c r="J78" s="20"/>
-      <c r="K78" s="20" t="str">
+        <v>24.9</v>
+      </c>
+      <c r="J78" s="20">
+        <v>48.63</v>
+      </c>
+      <c r="K78" s="20">
         <f t="shared" si="17"/>
-        <v/>
-      </c>
-      <c r="L78" s="13" t="str">
+        <v>81.67</v>
+      </c>
+      <c r="L78" s="13">
         <f>IF(OR($B78="",$C78=""),"",$C78*INDEX(Simulador!$F$7:$F$232,MATCH($B78,Simulador!$A$7:$A$232,0)))</f>
-        <v/>
-      </c>
-      <c r="M78" s="13" t="str">
+        <v>308.39999999999998</v>
+      </c>
+      <c r="M78" s="13">
         <f t="shared" si="13"/>
-        <v/>
-      </c>
-      <c r="N78" s="35" t="str">
+        <v>58.009000000000007</v>
+      </c>
+      <c r="N78" s="35">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="O78" s="12" t="str">
+        <v>108.28100000000001</v>
+      </c>
+      <c r="O78" s="12">
         <f t="shared" si="15"/>
-        <v/>
+        <v>0.18666241445292972</v>
       </c>
       <c r="P78" s="22" t="str">
         <f t="shared" si="16"/>
-        <v/>
+        <v>DENTRO DA META (15-20%)</v>
       </c>
       <c r="Q78" s="19"/>
       <c r="R78" s="19"/>
+      <c r="S78" t="s">
+        <v>560</v>
+      </c>
     </row>
     <row r="79" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="32"/>
@@ -21969,34 +22010,34 @@
       </c>
       <c r="G108" s="39">
         <f>SUM(G6:G107)</f>
-        <v>29059.240000000013</v>
+        <v>31278.350000000013</v>
       </c>
       <c r="K108" s="39">
         <f>SUM(K6:K107)</f>
-        <v>4433.4200000000019</v>
+        <v>4753.8800000000028</v>
       </c>
       <c r="L108" s="39">
         <f>SUM(L6:L107)</f>
-        <v>15252.43</v>
+        <v>16352.61</v>
       </c>
       <c r="M108" s="39">
         <f>SUM(M6:M107)</f>
-        <v>2905.924</v>
+        <v>3127.835</v>
       </c>
       <c r="N108" s="39">
         <f>SUM(N6:N107)</f>
-        <v>7395.0460000000003</v>
+        <v>7893.7150000000011</v>
       </c>
       <c r="O108" s="40">
         <f>IF(G108=0,"",N108/G108)</f>
-        <v>0.2544817414357704</v>
+        <v>0.25236992999950436</v>
       </c>
     </row>
     <row r="117" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A117" s="41"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="S6:S75">
+  <conditionalFormatting sqref="S6:S78">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"DEVOLUÇÃO"</formula>
     </cfRule>

</xml_diff>